<commit_message>
Add and update metadata and analysis files
Added Genus-normalised-metadata.csv and metadata.csv for expanded sample and genus-level data. Renamed Phenotype-manuscript.R to Phenotype-manuscript_clean.R for clarity. Updated Clinical_metadata_summarised.xlsx with new or revised clinical metadata.
</commit_message>
<xml_diff>
--- a/Clinical_metadata_summarised.xlsx
+++ b/Clinical_metadata_summarised.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/mteng_ic_ac_uk/Documents/Projects/Experiments/NT008_Phenotype/Original-files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mteng/Documents/GitHub/PHENOTYPE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{F562D896-0EFA-2D4C-900A-1852462ACD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A413813-E8D1-4046-B6C5-A057A7D7149B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3123E421-2C93-314B-8DF6-BE48390AF9F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-33120" yWindow="1260" windowWidth="31360" windowHeight="20340" xr2:uid="{0753D1ED-BA58-1B45-9BB6-5C3CDFB1CAD7}"/>
+    <workbookView xWindow="-33120" yWindow="2360" windowWidth="31360" windowHeight="20340" xr2:uid="{0753D1ED-BA58-1B45-9BB6-5C3CDFB1CAD7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="32">
   <si>
     <t>PHENOTYPE ID</t>
   </si>
@@ -105,13 +105,40 @@
   </si>
   <si>
     <t>Age</t>
+  </si>
+  <si>
+    <t>Ex-smoker</t>
+  </si>
+  <si>
+    <t>Non-smoker</t>
+  </si>
+  <si>
+    <t>Non smoker</t>
+  </si>
+  <si>
+    <t>Smoker</t>
+  </si>
+  <si>
+    <t>Smoking_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male </t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Sex</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -126,6 +153,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -135,7 +169,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -171,11 +205,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -190,6 +248,23 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -524,2166 +599,2424 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C72913-69A4-B24B-BAD8-06667A19EA08}">
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:S44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="8" width="10.83203125" style="1"/>
-    <col min="9" max="9" width="10.83203125" style="2"/>
-    <col min="10" max="10" width="10.83203125" style="1"/>
-    <col min="11" max="11" width="10.83203125" style="3"/>
-    <col min="12" max="12" width="23.6640625" style="4" customWidth="1"/>
-    <col min="13" max="17" width="10.83203125" style="1"/>
+    <col min="1" max="3" width="12.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.83203125" customWidth="1"/>
+    <col min="6" max="9" width="10.83203125" style="1"/>
+    <col min="10" max="10" width="10.83203125" style="2"/>
+    <col min="11" max="11" width="10.83203125" style="1"/>
+    <col min="12" max="12" width="10.83203125" style="3"/>
+    <col min="13" max="13" width="23.6640625" style="4" customWidth="1"/>
+    <col min="14" max="18" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:19" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="8" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="S1" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A2" s="9">
         <v>1001</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="9">
         <v>55</v>
       </c>
-      <c r="C2"/>
-      <c r="D2" t="s">
+      <c r="D2" s="9"/>
+      <c r="E2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E2">
+      <c r="F2" s="9">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G2">
+      <c r="H2" s="9">
         <v>4.3</v>
       </c>
-      <c r="H2">
+      <c r="I2" s="9">
         <v>0.8</v>
       </c>
-      <c r="I2">
+      <c r="J2" s="9">
         <v>146</v>
       </c>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2">
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9">
         <v>2.86</v>
       </c>
-      <c r="M2">
+      <c r="N2" s="9">
         <v>88</v>
       </c>
-      <c r="N2">
+      <c r="O2" s="9">
         <v>3.72</v>
       </c>
-      <c r="O2">
+      <c r="P2" s="9">
         <v>90</v>
       </c>
-      <c r="P2">
+      <c r="Q2" s="9">
         <v>8.41</v>
       </c>
-      <c r="Q2">
+      <c r="R2" s="9">
         <v>93</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="S2" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A3" s="9">
         <v>1007</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="9">
         <v>57</v>
       </c>
-      <c r="C3"/>
-      <c r="D3" t="s">
+      <c r="D3" s="9"/>
+      <c r="E3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E3">
+      <c r="F3" s="9">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G3">
+      <c r="H3" s="9">
         <v>3.9</v>
       </c>
-      <c r="H3">
+      <c r="I3" s="9">
         <v>1</v>
       </c>
-      <c r="I3">
+      <c r="J3" s="9">
         <v>92.9</v>
       </c>
-      <c r="J3">
+      <c r="K3" s="9">
         <v>553</v>
       </c>
-      <c r="K3">
+      <c r="L3" s="9">
         <v>5.54</v>
       </c>
-      <c r="L3">
+      <c r="M3" s="9">
         <v>3.9</v>
       </c>
-      <c r="M3">
+      <c r="N3" s="9">
         <v>96</v>
       </c>
-      <c r="N3">
+      <c r="O3" s="9">
         <v>4.8099999999999996</v>
       </c>
-      <c r="O3">
+      <c r="P3" s="9">
         <v>91</v>
       </c>
-      <c r="P3">
+      <c r="Q3" s="9">
         <v>10.15</v>
       </c>
-      <c r="Q3">
+      <c r="R3" s="9">
         <v>98</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="S3" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A4" s="9">
         <v>1024</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="9">
         <v>74</v>
       </c>
-      <c r="C4">
+      <c r="D4" s="9">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E4">
+      <c r="F4" s="9">
         <v>20</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G4">
+      <c r="H4" s="9">
         <v>9.6999999999999993</v>
       </c>
-      <c r="H4">
+      <c r="I4" s="9">
         <v>1.4</v>
       </c>
-      <c r="I4">
+      <c r="J4" s="9">
         <v>137.19999999999999</v>
       </c>
-      <c r="J4">
+      <c r="K4" s="9">
         <v>2286</v>
       </c>
-      <c r="K4">
+      <c r="L4" s="9">
         <v>7.34</v>
       </c>
-      <c r="L4">
+      <c r="M4" s="9">
         <v>1.75</v>
       </c>
-      <c r="M4">
+      <c r="N4" s="9">
         <v>111</v>
       </c>
-      <c r="N4">
+      <c r="O4" s="9">
         <v>2.14</v>
       </c>
-      <c r="O4">
+      <c r="P4" s="9">
         <v>106</v>
       </c>
-      <c r="P4">
+      <c r="Q4" s="9">
         <v>3.98</v>
       </c>
-      <c r="Q4">
+      <c r="R4" s="9">
         <v>76</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5">
+      <c r="S4" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A5" s="9">
         <v>1034</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="9">
         <v>70</v>
       </c>
-      <c r="C5">
+      <c r="D5" s="9">
         <v>5.3</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E5">
+      <c r="F5" s="9">
         <v>65</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G5">
+      <c r="H5" s="9">
         <v>10.4</v>
       </c>
-      <c r="H5">
+      <c r="I5" s="9">
         <v>0.6</v>
       </c>
-      <c r="I5">
+      <c r="J5" s="9">
         <v>308.39999999999998</v>
       </c>
-      <c r="J5">
+      <c r="K5" s="9">
         <v>745</v>
       </c>
-      <c r="K5">
+      <c r="L5" s="9">
         <v>8.56</v>
       </c>
-      <c r="L5">
+      <c r="M5" s="9">
         <v>3.57</v>
       </c>
-      <c r="M5">
+      <c r="N5" s="9">
         <v>112</v>
       </c>
-      <c r="N5">
+      <c r="O5" s="9">
         <v>4.09</v>
       </c>
-      <c r="O5">
+      <c r="P5" s="9">
         <v>97</v>
       </c>
-      <c r="P5">
+      <c r="Q5" s="9">
         <v>6.93</v>
       </c>
-      <c r="Q5">
+      <c r="R5" s="9">
         <v>81</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6">
+      <c r="S5" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A6" s="9">
         <v>1037</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="9">
         <v>74</v>
       </c>
-      <c r="C6">
+      <c r="D6" s="9">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E6">
+      <c r="F6" s="9">
         <v>10</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G6">
+      <c r="H6" s="9">
         <v>7.8</v>
       </c>
-      <c r="H6">
+      <c r="I6" s="9">
         <v>1.1000000000000001</v>
       </c>
-      <c r="I6">
+      <c r="J6" s="9">
         <v>177.5</v>
       </c>
-      <c r="J6">
+      <c r="K6" s="9">
         <v>691</v>
       </c>
-      <c r="K6">
+      <c r="L6" s="9">
         <v>6.21</v>
       </c>
-      <c r="L6">
+      <c r="M6" s="9">
         <v>2.31</v>
       </c>
-      <c r="M6">
+      <c r="N6" s="9">
         <v>114</v>
       </c>
-      <c r="N6">
+      <c r="O6" s="9">
         <v>2.79</v>
       </c>
-      <c r="O6">
+      <c r="P6" s="9">
         <v>106</v>
       </c>
-      <c r="P6">
+      <c r="Q6" s="9">
         <v>4</v>
       </c>
-      <c r="Q6">
+      <c r="R6" s="9">
         <v>64</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7">
+      <c r="S6" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A7" s="9">
         <v>1048</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="9">
         <v>55</v>
       </c>
-      <c r="C7">
+      <c r="D7" s="9">
         <v>2.2999999999999998</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E7">
+      <c r="F7" s="9">
         <v>70</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G7">
+      <c r="H7" s="9">
         <v>11.2</v>
       </c>
-      <c r="H7">
+      <c r="I7" s="9">
         <v>0.5</v>
       </c>
-      <c r="I7">
+      <c r="J7" s="9">
         <v>172.8</v>
       </c>
-      <c r="J7">
+      <c r="K7" s="9">
         <v>515</v>
       </c>
-      <c r="K7">
+      <c r="L7" s="9">
         <v>9.33</v>
       </c>
-      <c r="L7">
+      <c r="M7" s="9">
         <v>2.98</v>
       </c>
-      <c r="M7">
+      <c r="N7" s="9">
         <v>94</v>
       </c>
-      <c r="N7">
+      <c r="O7" s="9">
         <v>3.5</v>
       </c>
-      <c r="O7">
+      <c r="P7" s="9">
         <v>87</v>
       </c>
-      <c r="P7">
+      <c r="Q7" s="9">
         <v>8.5</v>
       </c>
-      <c r="Q7">
+      <c r="R7" s="9">
         <v>97</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8">
+      <c r="S7" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A8" s="9">
         <v>1051</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="9">
         <v>65</v>
       </c>
-      <c r="C8"/>
-      <c r="D8" t="s">
+      <c r="D8" s="9"/>
+      <c r="E8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E8">
+      <c r="F8" s="9">
         <v>75</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G8">
+      <c r="H8" s="9">
         <v>6.9</v>
       </c>
-      <c r="H8">
+      <c r="I8" s="9">
         <v>0.5</v>
       </c>
-      <c r="I8">
+      <c r="J8" s="9">
         <v>236.7</v>
       </c>
-      <c r="J8">
+      <c r="K8" s="9">
         <v>4983</v>
       </c>
-      <c r="K8">
+      <c r="L8" s="9">
         <v>8.33</v>
       </c>
-      <c r="L8">
+      <c r="M8" s="9">
         <v>2.56</v>
       </c>
-      <c r="M8">
+      <c r="N8" s="9">
         <v>95</v>
       </c>
-      <c r="N8">
+      <c r="O8" s="9">
         <v>3.09</v>
       </c>
-      <c r="O8">
+      <c r="P8" s="9">
         <v>89</v>
       </c>
-      <c r="P8">
+      <c r="Q8" s="9">
         <v>5.89</v>
       </c>
-      <c r="Q8">
+      <c r="R8" s="9">
         <v>76</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9">
+      <c r="S8" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A9" s="9">
         <v>1052</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="9">
         <v>52</v>
       </c>
-      <c r="C9"/>
-      <c r="D9" t="s">
+      <c r="D9" s="9"/>
+      <c r="E9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E9">
+      <c r="F9" s="9">
         <v>70</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G9">
+      <c r="H9" s="9">
         <v>1.6</v>
       </c>
-      <c r="H9">
+      <c r="I9" s="9">
         <v>0.7</v>
       </c>
-      <c r="I9">
+      <c r="J9" s="9">
         <v>354.4</v>
       </c>
-      <c r="J9">
+      <c r="K9" s="9">
         <v>1474</v>
       </c>
-      <c r="K9">
+      <c r="L9" s="9">
         <v>10.34</v>
       </c>
-      <c r="L9">
+      <c r="M9" s="9">
         <v>3.47</v>
       </c>
-      <c r="M9">
+      <c r="N9" s="9">
         <v>89</v>
       </c>
-      <c r="N9">
+      <c r="O9" s="9">
         <v>4.28</v>
       </c>
-      <c r="O9">
+      <c r="P9" s="9">
         <v>87</v>
       </c>
-      <c r="P9">
+      <c r="Q9" s="9">
         <v>9.3800000000000008</v>
       </c>
-      <c r="Q9">
+      <c r="R9" s="9">
         <v>96</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="S9" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A10" s="9">
         <v>1054</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="9">
         <v>66</v>
       </c>
-      <c r="C10">
+      <c r="D10" s="9">
         <v>3.3</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E10">
+      <c r="F10" s="9">
         <v>80</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G10">
+      <c r="H10" s="9">
         <v>12.7</v>
       </c>
-      <c r="H10">
+      <c r="I10" s="9">
         <v>0.8</v>
       </c>
-      <c r="I10">
+      <c r="J10" s="9">
         <v>312.2</v>
       </c>
-      <c r="J10">
+      <c r="K10" s="9">
         <v>491</v>
       </c>
-      <c r="K10">
+      <c r="L10" s="9">
         <v>10.52</v>
       </c>
-      <c r="L10">
+      <c r="M10" s="9">
         <v>1.55</v>
       </c>
-      <c r="M10">
+      <c r="N10" s="9">
         <v>92</v>
       </c>
-      <c r="N10">
+      <c r="O10" s="9">
         <v>1.67</v>
       </c>
-      <c r="O10">
+      <c r="P10" s="9">
         <v>78</v>
       </c>
-      <c r="P10">
+      <c r="Q10" s="9">
         <v>3.66</v>
       </c>
-      <c r="Q10">
+      <c r="R10" s="9">
         <v>71</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A11">
+      <c r="S10" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A11" s="9">
         <v>1060</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="9">
         <v>61</v>
       </c>
-      <c r="C11">
+      <c r="D11" s="9">
         <v>5.6</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E11">
+      <c r="F11" s="9">
         <v>75</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G11">
+      <c r="H11" s="9">
         <v>15.9</v>
       </c>
-      <c r="H11">
+      <c r="I11" s="9">
         <v>0.7</v>
       </c>
-      <c r="I11">
+      <c r="J11" s="9">
         <v>374.4</v>
       </c>
-      <c r="J11">
+      <c r="K11" s="9">
         <v>1950</v>
       </c>
-      <c r="K11">
+      <c r="L11" s="9">
         <v>9.6</v>
       </c>
-      <c r="L11">
+      <c r="M11" s="9">
         <v>3.05</v>
       </c>
-      <c r="M11">
+      <c r="N11" s="9">
         <v>100</v>
       </c>
-      <c r="N11">
+      <c r="O11" s="9">
         <v>3.53</v>
       </c>
-      <c r="O11">
+      <c r="P11" s="9">
         <v>90</v>
       </c>
-      <c r="P11">
+      <c r="Q11" s="9">
         <v>10.210000000000001</v>
       </c>
-      <c r="Q11">
+      <c r="R11" s="9">
         <v>119</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12">
+      <c r="S11" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A12" s="9">
         <v>1064</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="9">
         <v>49</v>
       </c>
-      <c r="C12">
+      <c r="D12" s="9">
         <v>0</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E12">
+      <c r="F12" s="9">
         <v>20</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G12">
+      <c r="H12" s="9">
         <v>6.1</v>
       </c>
-      <c r="H12">
+      <c r="I12" s="9">
         <v>0.7</v>
       </c>
-      <c r="I12">
+      <c r="J12" s="9">
         <v>367.4</v>
       </c>
-      <c r="J12">
+      <c r="K12" s="9">
         <v>6032</v>
       </c>
-      <c r="K12">
+      <c r="L12" s="9">
         <v>9.52</v>
       </c>
-      <c r="L12">
+      <c r="M12" s="9">
         <v>3.24</v>
       </c>
-      <c r="M12">
+      <c r="N12" s="9">
         <v>103</v>
       </c>
-      <c r="N12">
+      <c r="O12" s="9">
         <v>3.76</v>
       </c>
-      <c r="O12">
+      <c r="P12" s="9">
         <v>96</v>
       </c>
-      <c r="P12">
+      <c r="Q12" s="9">
         <v>8.59</v>
       </c>
-      <c r="Q12">
+      <c r="R12" s="9">
         <v>101</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A13">
+      <c r="S12" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A13" s="9">
         <v>1046</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="9">
         <v>56</v>
       </c>
-      <c r="C13">
+      <c r="D13" s="9">
         <v>2</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E13">
+      <c r="F13" s="9">
         <v>25</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G13">
+      <c r="H13" s="9">
         <v>5</v>
       </c>
-      <c r="H13">
+      <c r="I13" s="9">
         <v>1</v>
       </c>
-      <c r="I13">
+      <c r="J13" s="9">
         <v>199.7</v>
       </c>
-      <c r="J13">
+      <c r="K13" s="9">
         <v>677</v>
       </c>
-      <c r="K13">
+      <c r="L13" s="9">
         <v>8.09</v>
       </c>
-      <c r="L13"/>
-      <c r="M13"/>
-      <c r="N13"/>
-      <c r="O13"/>
-      <c r="P13"/>
-      <c r="Q13"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A14">
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9"/>
+      <c r="S13" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A14" s="9">
         <v>1063</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="9">
         <v>54</v>
       </c>
-      <c r="C14">
+      <c r="D14" s="9">
         <v>1.3</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E14">
+      <c r="F14" s="9">
         <v>20</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G14">
+      <c r="H14" s="9">
         <v>12.8</v>
       </c>
-      <c r="H14">
+      <c r="I14" s="9">
         <v>0.7</v>
       </c>
-      <c r="I14">
+      <c r="J14" s="9">
         <v>467.4</v>
       </c>
-      <c r="J14">
+      <c r="K14" s="9">
         <v>1562</v>
       </c>
-      <c r="K14">
+      <c r="L14" s="9">
         <v>9.31</v>
       </c>
-      <c r="L14">
+      <c r="M14" s="9">
         <v>3.77</v>
       </c>
-      <c r="M14">
+      <c r="N14" s="9">
         <v>107</v>
       </c>
-      <c r="N14">
+      <c r="O14" s="9">
         <v>4.1100000000000003</v>
       </c>
-      <c r="O14">
+      <c r="P14" s="9">
         <v>92</v>
       </c>
-      <c r="P14">
+      <c r="Q14" s="9">
         <v>10.25</v>
       </c>
-      <c r="Q14">
+      <c r="R14" s="9">
         <v>115</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A15">
+      <c r="S14" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A15" s="9">
         <v>1073</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="9">
         <v>65</v>
       </c>
-      <c r="C15">
+      <c r="D15" s="9">
         <v>2</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E15">
+      <c r="F15" s="9">
         <v>60</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G15"/>
-      <c r="H15"/>
-      <c r="I15"/>
-      <c r="J15"/>
-      <c r="K15"/>
-      <c r="L15">
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9">
         <v>3.56</v>
       </c>
-      <c r="M15">
+      <c r="N15" s="9">
         <v>124</v>
       </c>
-      <c r="N15">
+      <c r="O15" s="9">
         <v>3.9</v>
       </c>
-      <c r="O15">
+      <c r="P15" s="9">
         <v>109</v>
       </c>
-      <c r="P15">
+      <c r="Q15" s="9">
         <v>5.9</v>
       </c>
-      <c r="Q15">
+      <c r="R15" s="9">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A16">
+      <c r="S15" s="10"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A16" s="9">
         <v>1039</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="9">
         <v>83</v>
       </c>
-      <c r="C16">
+      <c r="D16" s="9">
         <v>5</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E16">
+      <c r="F16" s="9">
         <v>70</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G16">
+      <c r="H16" s="9">
         <v>10.1</v>
       </c>
-      <c r="H16">
+      <c r="I16" s="9">
         <v>0.4</v>
       </c>
-      <c r="I16">
+      <c r="J16" s="9">
         <v>232.6</v>
       </c>
-      <c r="J16">
+      <c r="K16" s="9">
         <v>534</v>
       </c>
-      <c r="K16">
+      <c r="L16" s="9">
         <v>4.78</v>
       </c>
-      <c r="L16">
+      <c r="M16" s="9">
         <v>1.95</v>
       </c>
-      <c r="M16">
+      <c r="N16" s="9">
         <v>98</v>
       </c>
-      <c r="N16">
+      <c r="O16" s="9">
         <v>2.2000000000000002</v>
       </c>
-      <c r="O16">
+      <c r="P16" s="9">
         <v>83</v>
       </c>
-      <c r="P16">
+      <c r="Q16" s="9">
         <v>4.53</v>
       </c>
-      <c r="Q16">
+      <c r="R16" s="9">
         <v>68</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A17">
+      <c r="S16" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A17" s="9">
         <v>1082</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="9">
         <v>52</v>
       </c>
-      <c r="C17">
+      <c r="D17" s="9">
         <v>1</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E17">
+      <c r="F17" s="9">
         <v>25</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G17">
+      <c r="H17" s="9">
         <v>9</v>
       </c>
-      <c r="H17">
+      <c r="I17" s="9">
         <v>0.4</v>
       </c>
-      <c r="I17">
+      <c r="J17" s="9">
         <v>261.89999999999998</v>
       </c>
-      <c r="J17">
+      <c r="K17" s="9">
         <v>418</v>
       </c>
-      <c r="K17">
+      <c r="L17" s="9">
         <v>8.77</v>
       </c>
-      <c r="L17">
+      <c r="M17" s="9">
         <v>3.83</v>
       </c>
-      <c r="M17">
+      <c r="N17" s="9">
         <v>117</v>
       </c>
-      <c r="N17">
+      <c r="O17" s="9">
         <v>4.6100000000000003</v>
       </c>
-      <c r="O17">
+      <c r="P17" s="9">
         <v>114</v>
       </c>
-      <c r="P17">
+      <c r="Q17" s="9">
         <v>7.61</v>
       </c>
-      <c r="Q17">
+      <c r="R17" s="9">
         <v>95</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A18">
+      <c r="S17" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A18" s="9">
         <v>1083</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="9">
         <v>58</v>
       </c>
-      <c r="C18">
+      <c r="D18" s="9">
         <v>14</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E18">
+      <c r="F18" s="9">
         <v>40</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G18">
+      <c r="H18" s="9">
         <v>18.100000000000001</v>
       </c>
-      <c r="H18">
+      <c r="I18" s="9">
         <v>0.6</v>
       </c>
-      <c r="I18">
+      <c r="J18" s="9">
         <v>345.4</v>
       </c>
-      <c r="J18">
+      <c r="K18" s="9">
         <v>2240</v>
       </c>
-      <c r="K18">
+      <c r="L18" s="9">
         <v>11.83</v>
       </c>
-      <c r="L18">
+      <c r="M18" s="9">
         <v>3.57</v>
       </c>
-      <c r="M18">
+      <c r="N18" s="9">
         <v>121</v>
       </c>
-      <c r="N18">
+      <c r="O18" s="9">
         <v>4</v>
       </c>
-      <c r="O18">
+      <c r="P18" s="9">
         <v>107</v>
       </c>
-      <c r="P18">
+      <c r="Q18" s="9">
         <v>6.4</v>
       </c>
-      <c r="Q18">
+      <c r="R18" s="9">
         <v>78</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A19">
+      <c r="S18" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A19" s="9">
         <v>1010</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="9">
         <v>54</v>
       </c>
-      <c r="C19">
+      <c r="D19" s="9">
         <v>0.7</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E19">
+      <c r="F19" s="9">
         <v>0</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G19">
+      <c r="H19" s="9">
         <v>6.7</v>
       </c>
-      <c r="H19">
+      <c r="I19" s="9">
         <v>1</v>
       </c>
-      <c r="I19">
+      <c r="J19" s="9">
         <v>154.19999999999999</v>
       </c>
-      <c r="J19">
+      <c r="K19" s="9">
         <v>1275</v>
       </c>
-      <c r="K19">
+      <c r="L19" s="9">
         <v>6.49</v>
       </c>
-      <c r="L19">
+      <c r="M19" s="9">
         <v>2.9</v>
       </c>
-      <c r="M19">
+      <c r="N19" s="9">
         <v>82</v>
       </c>
-      <c r="N19">
+      <c r="O19" s="9">
         <v>3.29</v>
       </c>
-      <c r="O19">
+      <c r="P19" s="9">
         <v>73</v>
       </c>
-      <c r="P19">
+      <c r="Q19" s="9">
         <v>7.26</v>
       </c>
-      <c r="Q19">
+      <c r="R19" s="9">
         <v>81</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A20">
+      <c r="S19" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A20" s="9">
         <v>1006</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="9">
         <v>46</v>
       </c>
-      <c r="C20">
+      <c r="D20" s="9">
         <v>4.3</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E20">
+      <c r="F20" s="9">
         <v>10</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G20">
+      <c r="H20" s="9">
         <v>7.6</v>
       </c>
-      <c r="H20">
+      <c r="I20" s="9">
         <v>0.8</v>
       </c>
-      <c r="I20">
+      <c r="J20" s="9">
         <v>147.19999999999999</v>
       </c>
-      <c r="J20">
+      <c r="K20" s="9">
         <v>1480</v>
       </c>
-      <c r="K20">
+      <c r="L20" s="9">
         <v>8.18</v>
       </c>
-      <c r="L20">
+      <c r="M20" s="9">
         <v>1.96</v>
       </c>
-      <c r="M20">
+      <c r="N20" s="9">
         <v>88</v>
       </c>
-      <c r="N20">
+      <c r="O20" s="9">
         <v>2.3199999999999998</v>
       </c>
-      <c r="O20">
+      <c r="P20" s="9">
         <v>85</v>
       </c>
-      <c r="P20">
+      <c r="Q20" s="9">
         <v>5.66</v>
       </c>
-      <c r="Q20">
+      <c r="R20" s="9">
         <v>94</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A21">
+      <c r="S20" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A21" s="9">
         <v>1095</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="9">
         <v>31</v>
       </c>
-      <c r="C21">
+      <c r="D21" s="9">
         <v>5.7</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E21">
+      <c r="F21" s="9">
         <v>0</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
-      <c r="J21"/>
-      <c r="K21"/>
-      <c r="L21">
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9">
         <v>4.57</v>
       </c>
-      <c r="M21">
+      <c r="N21" s="9">
         <v>98</v>
       </c>
-      <c r="N21">
+      <c r="O21" s="9">
         <v>5.66</v>
       </c>
-      <c r="O21">
+      <c r="P21" s="9">
         <v>100</v>
       </c>
-      <c r="P21">
+      <c r="Q21" s="9">
         <v>13.65</v>
       </c>
-      <c r="Q21">
+      <c r="R21" s="9">
         <v>120</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A22">
+      <c r="S21" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A22" s="9">
         <v>1036</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="9">
         <v>66</v>
       </c>
-      <c r="C22">
+      <c r="D22" s="9">
         <v>0</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E22">
+      <c r="F22" s="9">
         <v>20</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G22"/>
-      <c r="H22"/>
-      <c r="I22"/>
-      <c r="J22"/>
-      <c r="K22"/>
-      <c r="L22">
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9">
         <v>3.61</v>
       </c>
-      <c r="M22">
+      <c r="N22" s="9">
         <v>103</v>
       </c>
-      <c r="N22">
+      <c r="O22" s="9">
         <v>4.37</v>
       </c>
-      <c r="O22">
+      <c r="P22" s="9">
         <v>95</v>
       </c>
-      <c r="P22">
+      <c r="Q22" s="9">
         <v>9.8800000000000008</v>
       </c>
-      <c r="Q22">
+      <c r="R22" s="9">
         <v>107</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A23">
+      <c r="S22" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A23" s="9">
         <v>1106</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="9">
         <v>73</v>
       </c>
-      <c r="C23">
+      <c r="D23" s="9">
         <v>11</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E23">
+      <c r="F23" s="9">
         <v>35</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G23">
+      <c r="H23" s="9">
         <v>2.1</v>
       </c>
-      <c r="H23">
+      <c r="I23" s="9">
         <v>0.2</v>
       </c>
-      <c r="I23">
+      <c r="J23" s="9">
         <v>127.8</v>
       </c>
-      <c r="J23">
+      <c r="K23" s="9">
         <v>255</v>
       </c>
-      <c r="K23">
+      <c r="L23" s="9">
         <v>7.12</v>
       </c>
-      <c r="L23">
+      <c r="M23" s="9">
         <v>1.69</v>
       </c>
-      <c r="M23">
+      <c r="N23" s="9">
         <v>79</v>
       </c>
-      <c r="N23">
+      <c r="O23" s="9">
         <v>2.61</v>
       </c>
-      <c r="O23">
+      <c r="P23" s="9">
         <v>95</v>
       </c>
-      <c r="P23">
+      <c r="Q23" s="9">
         <v>3.58</v>
       </c>
-      <c r="Q23">
+      <c r="R23" s="9">
         <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A24">
+      <c r="S23" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A24" s="9">
         <v>1123</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" s="9">
         <v>62</v>
       </c>
-      <c r="C24">
+      <c r="D24" s="9">
         <v>5.7</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E24">
+      <c r="F24" s="9">
         <v>70</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G24">
+      <c r="H24" s="9">
         <v>14.7</v>
       </c>
-      <c r="H24">
+      <c r="I24" s="9">
         <v>0.3</v>
       </c>
-      <c r="I24">
+      <c r="J24" s="9">
         <v>75.400000000000006</v>
       </c>
-      <c r="J24">
+      <c r="K24" s="9">
         <v>1339</v>
       </c>
-      <c r="K24">
+      <c r="L24" s="9">
         <v>5.0999999999999996</v>
       </c>
-      <c r="L24">
+      <c r="M24" s="9">
         <v>3.28</v>
       </c>
-      <c r="M24">
+      <c r="N24" s="9">
         <v>91</v>
       </c>
-      <c r="N24">
+      <c r="O24" s="9">
         <v>4.0999999999999996</v>
       </c>
-      <c r="O24">
+      <c r="P24" s="9">
         <v>87</v>
       </c>
-      <c r="P24">
+      <c r="Q24" s="9">
         <v>3.19</v>
       </c>
-      <c r="Q24">
+      <c r="R24" s="9">
         <v>34</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A25">
+      <c r="S24" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A25" s="9">
         <v>1035</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="9">
         <v>70</v>
       </c>
-      <c r="C25">
+      <c r="D25" s="9">
         <v>0.5</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E25">
+      <c r="F25" s="9">
         <v>20</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G25">
+      <c r="H25" s="9">
         <v>3.4</v>
       </c>
-      <c r="H25">
+      <c r="I25" s="9">
         <v>0.9</v>
       </c>
-      <c r="I25">
+      <c r="J25" s="9">
         <v>41.4</v>
       </c>
-      <c r="J25"/>
-      <c r="K25">
+      <c r="K25" s="9"/>
+      <c r="L25" s="9">
         <v>3.35</v>
       </c>
-      <c r="L25"/>
-      <c r="M25"/>
-      <c r="N25"/>
-      <c r="O25"/>
-      <c r="P25"/>
-      <c r="Q25"/>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A26">
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A26" s="9">
         <v>1098</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" s="9">
         <v>75</v>
       </c>
-      <c r="C26">
+      <c r="D26" s="9">
         <v>1.3</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E26">
+      <c r="F26" s="9">
         <v>25</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G26">
+      <c r="H26" s="9">
         <v>17.100000000000001</v>
       </c>
-      <c r="H26">
+      <c r="I26" s="9">
         <v>0.8</v>
       </c>
-      <c r="I26">
+      <c r="J26" s="9">
         <v>117.2</v>
       </c>
-      <c r="J26">
+      <c r="K26" s="9">
         <v>2078</v>
       </c>
-      <c r="K26">
+      <c r="L26" s="9">
         <v>7.14</v>
       </c>
-      <c r="L26">
+      <c r="M26" s="9">
         <v>2.11</v>
       </c>
-      <c r="M26">
+      <c r="N26" s="9">
         <v>86</v>
       </c>
-      <c r="N26">
+      <c r="O26" s="9">
         <v>2.69</v>
       </c>
-      <c r="O26">
+      <c r="P26" s="9">
         <v>81</v>
       </c>
-      <c r="P26">
+      <c r="Q26" s="9">
         <v>5.17</v>
       </c>
-      <c r="Q26">
+      <c r="R26" s="9">
         <v>71</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A27">
+      <c r="S26" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A27" s="9">
         <v>1093</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="9">
         <v>30</v>
       </c>
-      <c r="C27">
+      <c r="D27" s="9">
         <v>0</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E27">
+      <c r="F27" s="9">
         <v>10</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G27">
+      <c r="H27" s="9">
         <v>25.3</v>
       </c>
-      <c r="H27">
+      <c r="I27" s="9">
         <v>0.6</v>
       </c>
-      <c r="I27">
+      <c r="J27" s="9">
         <v>310.10000000000002</v>
       </c>
-      <c r="J27">
+      <c r="K27" s="9">
         <v>948</v>
       </c>
-      <c r="K27">
+      <c r="L27" s="9">
         <v>7.45</v>
       </c>
-      <c r="L27">
+      <c r="M27" s="9">
         <v>2.69</v>
       </c>
-      <c r="M27">
+      <c r="N27" s="9">
         <v>102</v>
       </c>
-      <c r="N27">
+      <c r="O27" s="9">
         <v>2.96</v>
       </c>
-      <c r="O27">
+      <c r="P27" s="9">
         <v>96</v>
       </c>
-      <c r="P27">
+      <c r="Q27" s="9">
         <v>6.37</v>
       </c>
-      <c r="Q27">
+      <c r="R27" s="9">
         <v>96</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A28">
+      <c r="S27" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A28" s="9">
         <v>1100</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="9">
         <v>48</v>
       </c>
-      <c r="C28"/>
-      <c r="D28" t="s">
+      <c r="D28" s="9"/>
+      <c r="E28" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E28">
+      <c r="F28" s="9">
         <v>30</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G28">
+      <c r="H28" s="9">
         <v>9.3000000000000007</v>
       </c>
-      <c r="H28">
+      <c r="I28" s="9">
         <v>0.4</v>
       </c>
-      <c r="I28">
+      <c r="J28" s="9">
         <v>124.1</v>
       </c>
-      <c r="J28">
+      <c r="K28" s="9">
         <v>200</v>
       </c>
-      <c r="K28">
+      <c r="L28" s="9">
         <v>5.69</v>
       </c>
-      <c r="L28">
+      <c r="M28" s="9">
         <v>3.81</v>
       </c>
-      <c r="M28">
+      <c r="N28" s="9">
         <v>80</v>
       </c>
-      <c r="N28">
+      <c r="O28" s="9">
         <v>6.41</v>
       </c>
-      <c r="O28">
+      <c r="P28" s="9">
         <v>104</v>
       </c>
-      <c r="P28">
+      <c r="Q28" s="9">
         <v>6.25</v>
       </c>
-      <c r="Q28">
+      <c r="R28" s="9">
         <v>53</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A29">
+      <c r="S28" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A29" s="9">
         <v>1115</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="9">
         <v>48</v>
       </c>
-      <c r="C29">
+      <c r="D29" s="9">
         <v>1.7</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E29">
+      <c r="F29" s="9">
         <v>60</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G29">
+      <c r="H29" s="9">
         <v>7.3</v>
       </c>
-      <c r="H29">
+      <c r="I29" s="9">
         <v>0.4</v>
       </c>
-      <c r="I29">
+      <c r="J29" s="9">
         <v>164.9</v>
       </c>
-      <c r="J29">
+      <c r="K29" s="9">
         <v>4103</v>
       </c>
-      <c r="K29">
+      <c r="L29" s="9">
         <v>6.66</v>
       </c>
-      <c r="L29">
+      <c r="M29" s="9">
         <v>3.62</v>
       </c>
-      <c r="M29">
+      <c r="N29" s="9">
         <v>107</v>
       </c>
-      <c r="N29">
+      <c r="O29" s="9">
         <v>3.79</v>
       </c>
-      <c r="O29">
+      <c r="P29" s="9">
         <v>90</v>
       </c>
-      <c r="P29">
+      <c r="Q29" s="9">
         <v>7.2</v>
       </c>
-      <c r="Q29">
+      <c r="R29" s="9">
         <v>79</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A30">
+      <c r="S29" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A30" s="9">
         <v>1130</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="9">
         <v>32</v>
       </c>
-      <c r="C30"/>
-      <c r="D30" t="s">
+      <c r="D30" s="9"/>
+      <c r="E30" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E30">
+      <c r="F30" s="9">
         <v>40</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G30"/>
-      <c r="H30"/>
-      <c r="I30"/>
-      <c r="J30"/>
-      <c r="K30"/>
-      <c r="L30">
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9">
         <v>2.96</v>
       </c>
-      <c r="M30">
+      <c r="N30" s="9">
         <v>91</v>
       </c>
-      <c r="N30">
+      <c r="O30" s="9">
         <v>3.78</v>
       </c>
-      <c r="O30">
+      <c r="P30" s="9">
         <v>92</v>
       </c>
-      <c r="P30">
+      <c r="Q30" s="9">
         <v>5.89</v>
       </c>
-      <c r="Q30">
+      <c r="R30" s="9">
         <v>66</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A31">
+      <c r="S30" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A31" s="9">
         <v>1111</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="9">
         <v>75</v>
       </c>
-      <c r="C31">
+      <c r="D31" s="9">
         <v>0</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E31">
+      <c r="F31" s="9">
         <v>50</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G31"/>
-      <c r="H31"/>
-      <c r="I31"/>
-      <c r="J31"/>
-      <c r="K31"/>
-      <c r="L31">
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9"/>
+      <c r="M31" s="9">
         <v>2.85</v>
       </c>
-      <c r="M31">
+      <c r="N31" s="9">
         <v>98</v>
       </c>
-      <c r="N31">
+      <c r="O31" s="9">
         <v>3.74</v>
       </c>
-      <c r="O31">
+      <c r="P31" s="9">
         <v>96</v>
       </c>
-      <c r="P31">
+      <c r="Q31" s="9">
         <v>5.24</v>
       </c>
-      <c r="Q31">
+      <c r="R31" s="9">
         <v>65</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A32">
+      <c r="S31" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A32" s="9">
         <v>1129</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="9">
         <v>53</v>
       </c>
-      <c r="C32">
+      <c r="D32" s="9">
         <v>2</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E32">
+      <c r="F32" s="9">
         <v>0</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G32"/>
-      <c r="H32"/>
-      <c r="I32"/>
-      <c r="J32"/>
-      <c r="K32"/>
-      <c r="L32">
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+      <c r="M32" s="9">
         <v>3.89</v>
       </c>
-      <c r="M32">
+      <c r="N32" s="9">
         <v>100</v>
       </c>
-      <c r="N32">
+      <c r="O32" s="9">
         <v>4.95</v>
       </c>
-      <c r="O32">
+      <c r="P32" s="9">
         <v>100</v>
       </c>
-      <c r="P32">
+      <c r="Q32" s="9">
         <v>6.65</v>
       </c>
-      <c r="Q32">
+      <c r="R32" s="9">
         <v>68</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A33">
+      <c r="S32" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A33" s="9">
         <v>1181</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" s="9">
         <v>55</v>
       </c>
-      <c r="C33">
+      <c r="D33" s="9">
         <v>0.7</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E33">
+      <c r="F33" s="9">
         <v>80</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G33">
+      <c r="H33" s="9">
         <v>11.8</v>
       </c>
-      <c r="H33">
+      <c r="I33" s="9">
         <v>0.6</v>
       </c>
-      <c r="I33">
+      <c r="J33" s="9">
         <v>277.10000000000002</v>
       </c>
-      <c r="J33">
+      <c r="K33" s="9">
         <v>3221</v>
       </c>
-      <c r="K33">
+      <c r="L33" s="9">
         <v>8.9600000000000009</v>
       </c>
-      <c r="L33">
+      <c r="M33" s="9">
         <v>3.14</v>
       </c>
-      <c r="M33">
+      <c r="N33" s="9">
         <v>88</v>
       </c>
-      <c r="N33">
+      <c r="O33" s="9">
         <v>4.18</v>
       </c>
-      <c r="O33">
+      <c r="P33" s="9">
         <v>92</v>
       </c>
-      <c r="P33">
+      <c r="Q33" s="9">
         <v>6.32</v>
       </c>
-      <c r="Q33">
+      <c r="R33" s="9">
         <v>65</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A34">
+      <c r="S33" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A34" s="9">
         <v>1155</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="9">
         <v>53</v>
       </c>
-      <c r="C34">
+      <c r="D34" s="9">
         <v>1</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E34">
+      <c r="F34" s="9">
         <v>80</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G34">
+      <c r="H34" s="9">
         <v>12.2</v>
       </c>
-      <c r="H34">
+      <c r="I34" s="9">
         <v>0.4</v>
       </c>
-      <c r="I34">
+      <c r="J34" s="9">
         <v>194.7</v>
       </c>
-      <c r="J34">
+      <c r="K34" s="9">
         <v>1248</v>
       </c>
-      <c r="K34">
+      <c r="L34" s="9">
         <v>8.83</v>
       </c>
-      <c r="L34">
+      <c r="M34" s="9">
         <v>1.48</v>
       </c>
-      <c r="M34">
+      <c r="N34" s="9">
         <v>71</v>
       </c>
-      <c r="N34">
+      <c r="O34" s="9">
         <v>1.64</v>
       </c>
-      <c r="O34">
+      <c r="P34" s="9">
         <v>63</v>
       </c>
-      <c r="P34">
+      <c r="Q34" s="9">
         <v>3.75</v>
       </c>
-      <c r="Q34">
+      <c r="R34" s="9">
         <v>64</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A35">
+      <c r="S34" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A35" s="9">
         <v>1174</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="9">
         <v>63</v>
       </c>
-      <c r="C35">
+      <c r="D35" s="9">
         <v>0.67</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E35">
+      <c r="F35" s="9">
         <v>50</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G35">
+      <c r="H35" s="9">
         <v>12.1</v>
       </c>
-      <c r="H35">
+      <c r="I35" s="9">
         <v>0.5</v>
       </c>
-      <c r="I35">
+      <c r="J35" s="9">
         <v>102.4</v>
       </c>
-      <c r="J35">
+      <c r="K35" s="9">
         <v>4787</v>
       </c>
-      <c r="K35">
+      <c r="L35" s="9">
         <v>6.45</v>
       </c>
-      <c r="L35">
+      <c r="M35" s="9">
         <v>2.9</v>
       </c>
-      <c r="M35">
+      <c r="N35" s="9">
         <v>113</v>
       </c>
-      <c r="N35">
+      <c r="O35" s="9">
         <v>3.26</v>
       </c>
-      <c r="O35">
+      <c r="P35" s="9">
         <v>100</v>
       </c>
-      <c r="P35">
+      <c r="Q35" s="9">
         <v>7.39</v>
       </c>
-      <c r="Q35">
+      <c r="R35" s="9">
         <v>101</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A36">
+      <c r="S35" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A36" s="9">
         <v>1153</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="9">
         <v>63</v>
       </c>
-      <c r="C36">
+      <c r="D36" s="9">
         <v>0.33</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E36">
+      <c r="F36" s="9">
         <v>80</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G36">
+      <c r="H36" s="9">
         <v>16.7</v>
       </c>
-      <c r="H36">
+      <c r="I36" s="9">
         <v>1.2</v>
       </c>
-      <c r="I36">
+      <c r="J36" s="9">
         <v>162</v>
       </c>
-      <c r="J36">
+      <c r="K36" s="9">
         <v>705</v>
       </c>
-      <c r="K36">
+      <c r="L36" s="9">
         <v>7.95</v>
       </c>
-      <c r="L36">
+      <c r="M36" s="9">
         <v>2</v>
       </c>
-      <c r="M36">
+      <c r="N36" s="9">
         <v>69</v>
       </c>
-      <c r="N36">
+      <c r="O36" s="9">
         <v>2.12</v>
       </c>
-      <c r="O36">
+      <c r="P36" s="9">
         <v>56</v>
       </c>
-      <c r="P36">
+      <c r="Q36" s="9">
         <v>5.64</v>
       </c>
-      <c r="Q36">
+      <c r="R36" s="9">
         <v>68</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A37">
+      <c r="S36" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A37" s="9">
         <v>1146</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="9">
         <v>43</v>
       </c>
-      <c r="C37">
+      <c r="D37" s="9">
         <v>2</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E37">
+      <c r="F37" s="9">
         <v>20</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G37">
+      <c r="H37" s="9">
         <v>12</v>
       </c>
-      <c r="H37">
+      <c r="I37" s="9">
         <v>0.9</v>
       </c>
-      <c r="I37">
+      <c r="J37" s="9">
         <v>230.1</v>
       </c>
-      <c r="J37">
+      <c r="K37" s="9">
         <v>778</v>
       </c>
-      <c r="K37">
+      <c r="L37" s="9">
         <v>7.31</v>
       </c>
-      <c r="L37">
+      <c r="M37" s="9">
         <v>4.3499999999999996</v>
       </c>
-      <c r="M37">
+      <c r="N37" s="9">
         <v>100</v>
       </c>
-      <c r="N37">
+      <c r="O37" s="9">
         <v>5.07</v>
       </c>
-      <c r="O37">
+      <c r="P37" s="9">
         <v>93</v>
       </c>
-      <c r="P37">
+      <c r="Q37" s="9">
         <v>11.12</v>
       </c>
-      <c r="Q37">
+      <c r="R37" s="9">
         <v>104</v>
       </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A38">
+      <c r="S37" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A38" s="9">
         <v>1151</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" s="9">
         <v>76</v>
       </c>
-      <c r="C38">
+      <c r="D38" s="9">
         <v>0.3</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E38">
+      <c r="F38" s="9">
         <v>80</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G38">
+      <c r="H38" s="9">
         <v>18.899999999999999</v>
       </c>
-      <c r="H38">
+      <c r="I38" s="9">
         <v>0.7</v>
       </c>
-      <c r="I38">
+      <c r="J38" s="9">
         <v>441.5</v>
       </c>
-      <c r="J38">
+      <c r="K38" s="9">
         <v>3218</v>
       </c>
-      <c r="K38">
+      <c r="L38" s="9">
         <v>10.1</v>
       </c>
-      <c r="L38">
+      <c r="M38" s="9">
         <v>2.5</v>
       </c>
-      <c r="M38">
+      <c r="N38" s="9">
         <v>85</v>
       </c>
-      <c r="N38">
+      <c r="O38" s="9">
         <v>2.99</v>
       </c>
-      <c r="O38">
+      <c r="P38" s="9">
         <v>76</v>
       </c>
-      <c r="P38">
+      <c r="Q38" s="9">
         <v>5.57</v>
       </c>
-      <c r="Q38">
+      <c r="R38" s="9">
         <v>68</v>
       </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A39">
+      <c r="S38" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A39" s="9">
         <v>1193</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C39" s="9">
         <v>49</v>
       </c>
-      <c r="C39">
+      <c r="D39" s="9">
         <v>1.7</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E39">
+      <c r="F39" s="9">
         <v>85</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G39">
+      <c r="H39" s="9">
         <v>10.7</v>
       </c>
-      <c r="H39">
+      <c r="I39" s="9">
         <v>0.3</v>
       </c>
-      <c r="I39">
+      <c r="J39" s="9">
         <v>65.099999999999994</v>
       </c>
-      <c r="J39">
+      <c r="K39" s="9">
         <v>3081</v>
       </c>
-      <c r="K39">
+      <c r="L39" s="9">
         <v>4.43</v>
       </c>
-      <c r="L39">
+      <c r="M39" s="9">
         <v>2.14</v>
       </c>
-      <c r="M39">
+      <c r="N39" s="9">
         <v>83</v>
       </c>
-      <c r="N39">
+      <c r="O39" s="9">
         <v>2.38</v>
       </c>
-      <c r="O39">
+      <c r="P39" s="9">
         <v>75</v>
       </c>
-      <c r="P39">
+      <c r="Q39" s="9">
         <v>4.4000000000000004</v>
       </c>
-      <c r="Q39">
+      <c r="R39" s="9">
         <v>67</v>
       </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A40">
+      <c r="S39" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A40" s="9">
         <v>1175</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="9">
         <v>62</v>
       </c>
-      <c r="C40">
+      <c r="D40" s="9">
         <v>0.3</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E40">
+      <c r="F40" s="9">
         <v>65</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G40">
+      <c r="H40" s="9">
         <v>15.4</v>
       </c>
-      <c r="H40">
+      <c r="I40" s="9">
         <v>0.5</v>
       </c>
-      <c r="I40">
+      <c r="J40" s="9">
         <v>76.099999999999994</v>
       </c>
-      <c r="J40">
+      <c r="K40" s="9">
         <v>622</v>
       </c>
-      <c r="K40">
+      <c r="L40" s="9">
         <v>7.2</v>
       </c>
-      <c r="L40">
+      <c r="M40" s="9">
         <v>2.93</v>
       </c>
-      <c r="M40">
+      <c r="N40" s="9">
         <v>81</v>
       </c>
-      <c r="N40">
+      <c r="O40" s="9">
         <v>3.68</v>
       </c>
-      <c r="O40">
+      <c r="P40" s="9">
         <v>78</v>
       </c>
-      <c r="P40">
+      <c r="Q40" s="9">
         <v>8.81</v>
       </c>
-      <c r="Q40">
+      <c r="R40" s="9">
         <v>93</v>
       </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A41">
+      <c r="S40" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A41" s="9">
         <v>1172</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" s="9">
         <v>58</v>
       </c>
-      <c r="C41">
+      <c r="D41" s="9">
         <v>0.3</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E41">
+      <c r="F41" s="9">
         <v>75</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G41"/>
-      <c r="H41"/>
-      <c r="I41"/>
-      <c r="J41"/>
-      <c r="K41"/>
-      <c r="L41">
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+      <c r="J41" s="9"/>
+      <c r="K41" s="9"/>
+      <c r="L41" s="9"/>
+      <c r="M41" s="9">
         <v>3.54</v>
       </c>
-      <c r="M41">
+      <c r="N41" s="9">
         <v>124</v>
       </c>
-      <c r="N41">
+      <c r="O41" s="9">
         <v>3.71</v>
       </c>
-      <c r="O41">
+      <c r="P41" s="9">
         <v>102</v>
       </c>
-      <c r="P41">
+      <c r="Q41" s="9">
         <v>4.9800000000000004</v>
       </c>
-      <c r="Q41">
+      <c r="R41" s="9">
         <v>62</v>
       </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A42">
+      <c r="S41" s="12"/>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A42" s="9">
         <v>1189</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" s="9">
         <v>70</v>
       </c>
-      <c r="C42">
+      <c r="D42" s="9">
         <v>2.2999999999999998</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E42">
+      <c r="F42" s="9">
         <v>65</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G42"/>
-      <c r="H42"/>
-      <c r="I42"/>
-      <c r="J42"/>
-      <c r="K42"/>
-      <c r="L42">
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="9"/>
+      <c r="M42" s="9">
         <v>2.75</v>
       </c>
-      <c r="M42">
+      <c r="N42" s="9">
         <v>80.7</v>
       </c>
-      <c r="N42">
+      <c r="O42" s="9">
         <v>3.34</v>
       </c>
-      <c r="O42">
+      <c r="P42" s="9">
         <v>73.599999999999994</v>
       </c>
-      <c r="P42">
+      <c r="Q42" s="9">
         <v>5.64</v>
       </c>
-      <c r="Q42">
+      <c r="R42" s="9">
         <v>61.2</v>
       </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A43">
+      <c r="S42" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A43" s="9">
         <v>1170</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" s="9">
         <v>64</v>
       </c>
-      <c r="C43">
+      <c r="D43" s="9">
         <v>11</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E43">
+      <c r="F43" s="9">
         <v>70</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G43"/>
-      <c r="H43"/>
-      <c r="I43"/>
-      <c r="J43"/>
-      <c r="K43"/>
-      <c r="L43">
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="9"/>
+      <c r="M43" s="9">
         <v>2.5299999999999998</v>
       </c>
-      <c r="M43">
+      <c r="N43" s="9">
         <v>78</v>
       </c>
-      <c r="N43">
+      <c r="O43" s="9">
         <v>3.11</v>
       </c>
-      <c r="O43">
+      <c r="P43" s="9">
         <v>74</v>
       </c>
-      <c r="P43">
+      <c r="Q43" s="9">
         <v>3.7</v>
       </c>
-      <c r="Q43">
+      <c r="R43" s="9">
         <v>44</v>
       </c>
+      <c r="S43" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="J44" s="6"/>
+      <c r="M44" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>